<commit_message>
renamed a card, more images
</commit_message>
<xml_diff>
--- a/general_cards.xlsx
+++ b/general_cards.xlsx
@@ -54,10 +54,10 @@
     <t xml:space="preserve">Discard 3 and then draw up to your max hand size. Skip your next turn.</t>
   </si>
   <si>
-    <t>cardimages/burn_it.png</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Burn it</t>
+    <t>cardimages/refresh.png</t>
+  </si>
+  <si>
+    <t>Refresh</t>
   </si>
   <si>
     <t xml:space="preserve">Exhaust X cards from your hand. Draw X cards.</t>
@@ -201,7 +201,7 @@
     <t>cardimages/all_for_one.png</t>
   </si>
   <si>
-    <t xml:space="preserve">All for One/One for All</t>
+    <t xml:space="preserve">All for One</t>
   </si>
   <si>
     <t xml:space="preserve">Deal 10 Damage to the Monster, Prevent 10 Damage, then exile this card. If this card is discarded, Gather 1.</t>
@@ -741,7 +741,7 @@
   <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
     <col bestFit="1" min="1" max="1" width="35.28125"/>
-    <col bestFit="1" customWidth="1" min="2" max="2" width="19.28125"/>
+    <col bestFit="1" customWidth="1" min="2" max="2" width="19.80078125"/>
     <col bestFit="1" min="3" max="3" width="126.7109375"/>
   </cols>
   <sheetData>

</xml_diff>